<commit_message>
Add dashboard module insights and evidence-based viral report analysis
</commit_message>
<xml_diff>
--- a/examples/demo-output/demo-weekly.xlsx
+++ b/examples/demo-output/demo-weekly.xlsx
@@ -20,6 +20,8 @@
     <sheet name="趋势口径与查询" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="红人扩展档案" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="内容方向变化" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="模块分析与总结" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="爆款深度分析" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'口径与覆盖'!$A$1:$B$19</definedName>
@@ -35,6 +37,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'趋势口径与查询'!$A$1:$M$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'红人扩展档案'!$A$1:$Q$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'内容方向变化'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'模块分析与总结'!$A$1:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'爆款深度分析'!$A$1:$N$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -517,7 +521,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.277997+00:00</t>
+          <t>2026-10-30T02:27:13.886997+00:00</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1141,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263834+00:00</t>
+          <t>2026-10-30T02:27:13.875255+00:00</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -1194,7 +1198,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263908+00:00</t>
+          <t>2026-10-30T02:27:13.875331+00:00</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -1251,7 +1255,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263929+00:00</t>
+          <t>2026-10-30T02:27:13.875350+00:00</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -1308,7 +1312,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263943+00:00</t>
+          <t>2026-10-30T02:27:13.875364+00:00</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -1365,7 +1369,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263955+00:00</t>
+          <t>2026-10-30T02:27:13.875377+00:00</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1422,7 +1426,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263966+00:00</t>
+          <t>2026-10-30T02:27:13.875390+00:00</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1479,7 +1483,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263977+00:00</t>
+          <t>2026-10-30T02:27:13.875400+00:00</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1536,7 +1540,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263988+00:00</t>
+          <t>2026-10-30T02:27:13.875412+00:00</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1593,7 +1597,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.263998+00:00</t>
+          <t>2026-10-30T02:27:13.875424+00:00</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1650,7 +1654,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.264010+00:00</t>
+          <t>2026-10-30T02:27:13.875436+00:00</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1707,7 +1711,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.264020+00:00</t>
+          <t>2026-10-30T02:27:13.875449+00:00</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1764,7 +1768,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.264033+00:00</t>
+          <t>2026-10-30T02:27:13.875460+00:00</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1937,12 +1941,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -2020,12 +2024,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -2119,6 +2123,627 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>模块</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>数据事实</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>分析与总结</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Qronge行动（待验证）</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>限制</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>依据链接</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>本周动态分析与总结</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>选定统计范围本周发布 1 条，涉及 1 个平台账号；较上周 0 条变化 +1 条；从 0 增至 1。
+同范围本周发现 0 条、更新 1 条；疑似合作 1 条和官方内容 0 条单独展示。
+已收录数量变化分布：Yozma +1 条。这是样本构成变化，不是投放策略的因果解释；多品牌视频可能重复进入品牌分布。</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>发布数量变化只描述已收录、已审核样本，不足以判断竞品投放预算或策略变化。</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>优先审核合作证据、所在地与形式；将补录旧片保留为本周发现，不计新上线。</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>按顶部周、品牌、平台、车型和形式筛选；页面内文本搜索仅缩小明细，不改变这些汇总。
+疑似/官方计数来自视频列表，与选定合作汇总范围不同，不相加为确认合作。</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>品牌与车型分布解读</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>本周品牌发布分布：Yozma 1 条。
+本周车型标签分布：IN-10 Pro 1 条。</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>当前样本中出现最多的是 Yozma，覆盖 1/1 条发布记录。分布反映当前样本覆盖，不能据此推断竞品车型销量或合作费用。</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>对集中出现的车型补查产品版本、合作证据和创作者类型，形成Qronge选题对照。</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>同片出现多品牌/车型会分别进入标签分布，不应相加当去重视频数。</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>内容方向与标题分析</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>主要方向：评测 1 条，占 100%，较上周变化 +100 个百分点。
+原标题高频词：yozma、in-10、pro、review。</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>方向标签是系统归纳，标题词是原标题中的真实词；频次不等于选题效果或爆款成因。</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>将高频主题与同龄表现交叉复核，再安排Qronge选题测试；不只模仿标题词。</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>多标签占比可超过100%；未取得视频材料时不能判断封面、开场或结构。</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>曝光表现分析与总结</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>新上线内容已知累计播放 80,000，覆盖 1/1 条；均值 80,000，中位数 80,000。
+选定范围 0/2 条有可用增长窗口；历史内容观测区间增量 不可用。
+单条最高播放占已知播放的 100.0%（1 条有播放数据）。缺失指标未计入分母，不等于整体受众集中度。</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>当前累计播放只能作为曝光代理；缺失指标和不同视频年龄会影响均值、中位数及比较。</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>先补齐缺失快照，长短视频分组比较；优先采用发布后7天或30天的同龄表现。</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>没有基线不计算新增；观察窗口可能跨周界。跨平台播放量未去重受众。</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>视频监控分析与审核重点</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>视频列表收录 3 条非基线记录；其中本周发布 2、本周发现 0、本周更新 2，三个集合可重叠。
+待核实商业线索 1 条，所在地未知 1 条，观察截止点数据过期 1 条。</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>视频列表包含各种合作状态，数量不能直接当作已确认合作量。</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>先复核有披露、折扣码或联盟链接的记录，再核对国家与形式；对过期记录检查采集日志。</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>按顶部周、品牌、平台、车型和形式筛选；页面内文本搜索仅缩小明细，不改变这些汇总。
+本模块覆盖视频列表所有状态；选定合作指标见周度总览。</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>[DEMO] Tuttio Soleil01 GB Pro off-road first ride https://www.youtube.com/watch?v=demoNEW0002</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>爆款候选分析与总结</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>当前视频列表有 2 条候选：绝对高播放 1 条，相对账号爆款候选 1 条，两类可重叠。
+其中本周新上线 1 条、历史内容 1 条。</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>优先复核同龄基线充分的相对候选；绝对高播放不能替代相对异常判定。</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>逐条查看合作证据、实际观察窗口和材料来源；将可验证选题和创作者机会纳入下周研究清单。</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>候选覆盖当前视频列表非排除内容，并不只限选定合作状态或目标市场；卡片会单独标明。</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>搜索趋势分析与总结</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>当前周有 1 条完整周指数、0 条部分周记录；可比上周的上升记录 1 条。
+上升词：Yozma +6%（US/web，系列 DEMO-shared-normalization）。</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>变化只代表各查询自身在相同归一化批次内的相对热度，不能直接归因于红人合作。</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>补齐同地区、同渠道、同查询范围的12周指数和相关查询；把搜索变化与发布时间并列观察。</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>不相加跨批次指数；零基数不算百分比；缺失不补0。搜索渠道独立于视频平台筛选。</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Yozma DEMO合成趋势</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>红人库分析与合作机会</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>当前账号库 2 个平台账号，含确认合作记录 2 个，已有公开商务联系方式及来源 0 个，已关注 0 个。
+有爆款候选记录的账号 2 个；这不代表其全部内容的爆款率。</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>可先复核有候选表现和定位匹配的账号，粉丝规模或单条高播放不足以确定合作价值。</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>核对美国受众依据、同龄样本、内容类型和公开商务入口；保留低表现及暂无合作的账号供后续筛选。</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>账号库按平台/品牌筛选，保留历史档案；不等同于本周新合作名单。身份未经核实不跨平台合并。</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>采集覆盖分析与下一步</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>最近任务：尚无运行记录。
+最近展示的 0 条查询记录中，页数截断 0 条、失败 0 条。</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>接口成功只验证对应查询，不代表三平台全量覆盖；任务记录也不证明常驻进程仍在运行。</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>对失败和截断查询先查日志与配额；补录未接自动接口的平台数据，并定期验证本机夜间进程。</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Instagram/TikTok与Google Trends自动接口未接通；数据量不足时保留限制说明。</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>视频</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>原标题</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>候选类型</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>上线范围</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>合作状态</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>国家</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>语言</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>入选事实</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>内容观察</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>待核验推测</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>材料状态与来源</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>总结</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Qronge行动</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>分析限制</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=demoREL0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>[DEMO] Yozma IN-10 Pro review</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>相对爆款候选</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>历史内容复查</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>明确合作</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>相对爆款候选；历史视频；合作状态：明确合作。
+最后有效展示快照：2026-10-16T07:00:00+00:00，播放 400，点赞 100，评论 10，分享 不可用。
+发布后 7 天：同账号同形式 10 条可比样本中位数 100.0，本片为基线 4 倍。
+增长速度不可用：尚无有效的两次观测窗口，累计播放不视为本周新增。</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>原标题：[DEMO] Yozma IN-10 Pro review
+原标题品牌词：Yozma；车型词：IN-10 Pro。
+归纳主题标签（不等于原标题原词）：评测。</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>无附加推测</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">封面：不可用，未取得对应材料  
+开场：不可用，未取得对应材料  
+测试场景：不可用，未取得对应材料  
+内容结构：不可用，未取得对应材料  
+观众讨论点：不可用，未取得对应材料  
+字幕/口播：不可用，未取得对应材料  </t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>同龄可比指标支持其相对账号表现突出。现有指标不能证明传播原因、自然流量比例或转化效果。</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Qronge选题验证：以适用人群、实际体验和优缺点清单组织评测，先复核原片的评测维度。
+创作者机会：复核 DEMO同龄样本账号 的美国受众、内容定位及同龄历史表现；通过已记录的公开商务入口评估合作，不自动联系或推算报价。
+补录带来源的封面、开场、场景、结构和评论观察，未取得前不下内容因果结论。</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>未取得的材料不分析；人工备注与系统直接读取指标分开。
+候选清单包含已收录非排除内容，逐条标注合作状态与市场；不自动计入已确认合作。
+高播放不等于高转化，不推断订单、销售额、ROI或合作费用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=demoNEW0001</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>[DEMO] Yozma IN-10 Pro review</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>高播放视频</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>本周新上线</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>明确合作</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>高播放视频；本周发布；合作状态：明确合作。
+最后有效展示快照：2026-10-26T06:00:00+00:00，播放 80,000，点赞 100，评论 10，分享 不可用。
+达到 YouTube / YouTube 普通视频 的高播放阈值 50,000。
+同龄样本 0 条；样本不足/格式未知/缺少同龄快照，不计算精确倍数。
+增长速度不可用：尚无有效的两次观测窗口，累计播放不视为本周新增。</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>原标题：[DEMO] Yozma IN-10 Pro review
+原标题品牌词：Yozma；车型词：IN-10 Pro。
+归纳主题标签（不等于原标题原词）：评测。</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>无附加推测</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">封面：不可用，未取得对应材料  
+开场：不可用，未取得对应材料  
+测试场景：不可用，未取得对应材料  
+内容结构：不可用，未取得对应材料  
+观众讨论点：不可用，未取得对应材料  
+字幕/口播：不可用，未取得对应材料  </t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>目前只满足绝对高播放标准，尚不足以认定相对账号表现异常。现有指标不能证明传播原因、自然流量比例或转化效果。</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Qronge选题验证：以适用人群、实际体验和优缺点清单组织评测，先复核原片的评测维度。
+创作者机会：复核 DEMO测试账号 的美国受众、内容定位及同龄历史表现；通过已记录的公开商务入口评估合作，不自动联系或推算报价。
+补齐同账号最近10–12条同形式视频的同龄快照，再判断是否相对爆款。
+补录带来源的封面、开场、场景、结构和评论观察，未取得前不下内容因果结论。</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>未取得的材料不分析；人工备注与系统直接读取指标分开。
+候选清单包含已收录非排除内容，逐条标注合作状态与市场；不自动计入已确认合作。
+高播放不等于高转化，不推断订单、销售额、ROI或合作费用。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2329,7 +2954,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -2446,7 +3071,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -2734,7 +3359,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -2851,7 +3476,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -2970,7 +3595,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:51:57.257059+00:00</t>
+          <t>2026-10-30T02:27:13.868992+00:00</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Prioritize discount and affiliate evidence, apply 1000-view gate, simplify weekly report
</commit_message>
<xml_diff>
--- a/examples/demo-output/demo-weekly.xlsx
+++ b/examples/demo-output/demo-weekly.xlsx
@@ -15,30 +15,28 @@
     <sheet name="搜索趋势" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="周度汇总" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="品牌平台车型" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="爆款分析" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="爆款视频" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="效果与观察期" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="趋势口径与查询" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="红人扩展档案" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="内容方向变化" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="模块分析与总结" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="爆款深度分析" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="关键信号" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'口径与覆盖'!$A$1:$B$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'口径与覆盖'!$A$1:$B$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'本周发布视频'!$A$1:$Y$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'历史视频与效果'!$A$1:$Y$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'长短视频汇总'!$A$1:$E$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'红人名单'!$A$1:$J$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'搜索趋势'!$A$1:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'周度汇总'!$A$1:$B$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'周度汇总'!$A$1:$B$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'品牌平台车型'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'爆款分析'!$A$1:$S$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'爆款视频'!$A$1:$E$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'效果与观察期'!$A$1:$N$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'趋势口径与查询'!$A$1:$M$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'红人扩展档案'!$A$1:$Q$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'内容方向变化'!$A$1:$D$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'模块分析与总结'!$A$1:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'爆款深度分析'!$A$1:$N$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'关键信号'!$A$1:$A$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,10 +456,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -521,14 +519,14 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.886997+00:00</t>
+          <t>2026-10-30T02:55:55.482378+00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>美国英语已确认新合作视频</t>
+          <t>合作视频（折扣/联盟商业关联或人工确认）</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -548,125 +546,125 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>已知累计播放</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>80000</v>
+          <t>统计门槛</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>播放量≥1,000；未知播放待补；历史周按当时快照判断</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>播放量覆盖</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>1/1 条视频</t>
-        </is>
+          <t>已知累计播放</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>80000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>累计播放含义</t>
+          <t>播放量覆盖</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>本周新发布、已确认合作、美国英语视频在周末前最后一次快照的播放量；非去重触达</t>
+          <t>1/1 条视频</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>新增播放</t>
+          <t>累计播放含义</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>仅提供两次真实观测间的增量及起止时间；没有基线则留空，不推算整周</t>
+          <t>本周新发布、已确认合作、美国英语视频在周末前最后一次快照的播放量；非去重触达</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>历史覆盖</t>
+          <t>新增播放</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>目标近90天；首次采集无法恢复过去逐日播放量；导入/查询结果不代表全网总量</t>
+          <t>仅提供两次真实观测间的增量及起止时间；没有基线则留空，不推算整周</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>独立内容</t>
+          <t>历史覆盖</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>仅在人工提供 content_group 时跨平台合并，未提供时按独立发布计</t>
+          <t>目标近90天；首次采集无法恢复过去逐日播放量；导入/查询结果不代表全网总量</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>搜索趋势</t>
+          <t>独立内容</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>美国 Google Web 相对热度0–100；同 series_id 同 query 相邻完整周比较；非绝对搜索量</t>
+          <t>仅在人工提供 content_group 时跨平台合并，未提供时按独立发布计</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>爆款候选</t>
+          <t>搜索趋势</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>按平台内内容格式的绝对播放阈值筛选；不代表因果分析或保证自然流量</t>
+          <t>美国 Google Web 相对热度0–100；同 series_id 同 query 相邻完整周比较；非绝对搜索量</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>youtube</t>
+          <t>爆款候选</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>已配置凭据；详见运行结果</t>
+          <t>按平台内内容格式的绝对播放阈值筛选；不代表因果分析或保证自然流量</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>instagram</t>
+          <t>youtube</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>仅导入</t>
+          <t>已配置凭据；详见运行结果</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>tiktok</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -678,17 +676,29 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>仅导入</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>trends</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CSV导入；相关查询未导入则不可用</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B19"/>
+  <autoFilter ref="A1:B20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -811,10 +821,8 @@
           <t>不可用</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>不可用</t>
-        </is>
+      <c r="E2" t="n">
+        <v>4.4</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -950,7 +958,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>27.5</v>
+        <v>2.75</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -963,7 +971,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>400</v>
+        <v>4000</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -1141,7 +1149,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875255+00:00</t>
+          <t>2026-10-30T02:55:55.467409+00:00</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -1198,7 +1206,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875331+00:00</t>
+          <t>2026-10-30T02:55:55.467484+00:00</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -1255,7 +1263,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875350+00:00</t>
+          <t>2026-10-30T02:55:55.467503+00:00</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -1312,7 +1320,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875364+00:00</t>
+          <t>2026-10-30T02:55:55.467517+00:00</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -1369,7 +1377,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875377+00:00</t>
+          <t>2026-10-30T02:55:55.467529+00:00</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1426,7 +1434,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875390+00:00</t>
+          <t>2026-10-30T02:55:55.467542+00:00</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1483,7 +1491,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875400+00:00</t>
+          <t>2026-10-30T02:55:55.467554+00:00</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1540,7 +1548,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875412+00:00</t>
+          <t>2026-10-30T02:55:55.467564+00:00</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1597,7 +1605,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875424+00:00</t>
+          <t>2026-10-30T02:55:55.467627+00:00</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1654,7 +1662,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875436+00:00</t>
+          <t>2026-10-30T02:55:55.467638+00:00</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1711,7 +1719,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875449+00:00</t>
+          <t>2026-10-30T02:55:55.467649+00:00</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1768,7 +1776,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.875460+00:00</t>
+          <t>2026-10-30T02:55:55.467660+00:00</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1941,12 +1949,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -2024,19 +2032,19 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="K3" t="n">
         <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="M3" t="n">
         <v>1</v>
@@ -2133,617 +2141,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="47" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>模块</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>数据事实</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>分析与总结</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Qronge行动（待验证）</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>限制</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>依据链接</t>
+          <t>信号</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>本周动态分析与总结</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>选定统计范围本周发布 1 条，涉及 1 个平台账号；较上周 0 条变化 +1 条；从 0 增至 1。
-同范围本周发现 0 条、更新 1 条；疑似合作 1 条和官方内容 0 条单独展示。
-已收录数量变化分布：Yozma +1 条。这是样本构成变化，不是投放策略的因果解释；多品牌视频可能重复进入品牌分布。</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>发布数量变化只描述已收录、已审核样本，不足以判断竞品投放预算或策略变化。</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>优先审核合作证据、所在地与形式；将补录旧片保留为本周发现，不计新上线。</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>按顶部周、品牌、平台、车型和形式筛选；页面内文本搜索仅缩小明细，不改变这些汇总。
-疑似/官方计数来自视频列表，与选定合作汇总范围不同，不相加为确认合作。</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
+          <t>合作发布 1 条，1 个平台账号；较上周变化 +1 条。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>品牌与车型分布解读</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>本周品牌发布分布：Yozma 1 条。
-本周车型标签分布：IN-10 Pro 1 条。</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>当前样本中出现最多的是 Yozma，覆盖 1/1 条发布记录。分布反映当前样本覆盖，不能据此推断竞品车型销量或合作费用。</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>对集中出现的车型补查产品版本、合作证据和创作者类型，形成Qronge选题对照。</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>同片出现多品牌/车型会分别进入标签分布，不应相加当去重视频数。</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
+          <t>主要车型：IN-10 Pro 1条。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>内容方向与标题分析</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>主要方向：评测 1 条，占 100%，较上周变化 +100 个百分点。
-原标题高频词：yozma、in-10、pro、review。</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>方向标签是系统归纳，标题词是原标题中的真实词；频次不等于选题效果或爆款成因。</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>将高频主题与同龄表现交叉复核，再安排Qronge选题测试；不只模仿标题词。</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>多标签占比可超过100%；未取得视频材料时不能判断封面、开场或结构。</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>曝光表现分析与总结</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>新上线内容已知累计播放 80,000，覆盖 1/1 条；均值 80,000，中位数 80,000。
-选定范围 0/2 条有可用增长窗口；历史内容观测区间增量 不可用。
-单条最高播放占已知播放的 100.0%（1 条有播放数据）。缺失指标未计入分母，不等于整体受众集中度。</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>当前累计播放只能作为曝光代理；缺失指标和不同视频年龄会影响均值、中位数及比较。</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>先补齐缺失快照，长短视频分组比较；优先采用发布后7天或30天的同龄表现。</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>没有基线不计算新增；观察窗口可能跨周界。跨平台播放量未去重受众。</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>[DEMO] Yozma IN-10 Pro review https://www.youtube.com/watch?v=demoNEW0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>视频监控分析与审核重点</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>视频列表收录 3 条非基线记录；其中本周发布 2、本周发现 0、本周更新 2，三个集合可重叠。
-待核实商业线索 1 条，所在地未知 1 条，观察截止点数据过期 1 条。</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>视频列表包含各种合作状态，数量不能直接当作已确认合作量。</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>先复核有披露、折扣码或联盟链接的记录，再核对国家与形式；对过期记录检查采集日志。</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>按顶部周、品牌、平台、车型和形式筛选；页面内文本搜索仅缩小明细，不改变这些汇总。
-本模块覆盖视频列表所有状态；选定合作指标见周度总览。</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>[DEMO] Tuttio Soleil01 GB Pro off-road first ride https://www.youtube.com/watch?v=demoNEW0002</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>爆款候选分析与总结</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>当前视频列表有 2 条候选：绝对高播放 1 条，相对账号爆款候选 1 条，两类可重叠。
-其中本周新上线 1 条、历史内容 1 条。</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>优先复核同龄基线充分的相对候选；绝对高播放不能替代相对异常判定。</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>逐条查看合作证据、实际观察窗口和材料来源；将可验证选题和创作者机会纳入下周研究清单。</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>候选覆盖当前视频列表非排除内容，并不只限选定合作状态或目标市场；卡片会单独标明。</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>搜索趋势分析与总结</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>当前周有 1 条完整周指数、0 条部分周记录；可比上周的上升记录 1 条。
-上升词：Yozma +6%（US/web，系列 DEMO-shared-normalization）。</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>变化只代表各查询自身在相同归一化批次内的相对热度，不能直接归因于红人合作。</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>补齐同地区、同渠道、同查询范围的12周指数和相关查询；把搜索变化与发布时间并列观察。</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>不相加跨批次指数；零基数不算百分比；缺失不补0。搜索渠道独立于视频平台筛选。</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Yozma DEMO合成趋势</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>红人库分析与合作机会</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>当前账号库 2 个平台账号，含确认合作记录 2 个，已有公开商务联系方式及来源 0 个，已关注 0 个。
-有爆款候选记录的账号 2 个；这不代表其全部内容的爆款率。</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>可先复核有候选表现和定位匹配的账号，粉丝规模或单条高播放不足以确定合作价值。</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>核对美国受众依据、同龄样本、内容类型和公开商务入口；保留低表现及暂无合作的账号供后续筛选。</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>账号库按平台/品牌筛选，保留历史档案；不等同于本周新合作名单。身份未经核实不跨平台合并。</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>采集覆盖分析与下一步</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>最近任务：尚无运行记录。
-最近展示的 0 条查询记录中，页数截断 0 条、失败 0 条。</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>接口成功只验证对应查询，不代表三平台全量覆盖；任务记录也不证明常驻进程仍在运行。</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>对失败和截断查询先查日志与配额；补录未接自动接口的平台数据，并定期验证本机夜间进程。</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Instagram/TikTok与Google Trends自动接口未接通；数据量不足时保留限制说明。</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>达标爆款候选 2 条，其中本周发布 1 条，历史视频 1 条。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F10"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>视频</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>原标题</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>候选类型</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>上线范围</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>合作状态</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>国家</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>语言</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>入选事实</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>内容观察</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>待核验推测</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>材料状态与来源</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>总结</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Qronge行动</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>分析限制</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=demoREL0001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>[DEMO] Yozma IN-10 Pro review</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>相对爆款候选</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>历史内容复查</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>明确合作</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>相对爆款候选；历史视频；合作状态：明确合作。
-最后有效展示快照：2026-10-16T07:00:00+00:00，播放 400，点赞 100，评论 10，分享 不可用。
-发布后 7 天：同账号同形式 10 条可比样本中位数 100.0，本片为基线 4 倍。
-增长速度不可用：尚无有效的两次观测窗口，累计播放不视为本周新增。</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>原标题：[DEMO] Yozma IN-10 Pro review
-原标题品牌词：Yozma；车型词：IN-10 Pro。
-归纳主题标签（不等于原标题原词）：评测。</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>无附加推测</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">封面：不可用，未取得对应材料  
-开场：不可用，未取得对应材料  
-测试场景：不可用，未取得对应材料  
-内容结构：不可用，未取得对应材料  
-观众讨论点：不可用，未取得对应材料  
-字幕/口播：不可用，未取得对应材料  </t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>同龄可比指标支持其相对账号表现突出。现有指标不能证明传播原因、自然流量比例或转化效果。</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Qronge选题验证：以适用人群、实际体验和优缺点清单组织评测，先复核原片的评测维度。
-创作者机会：复核 DEMO同龄样本账号 的美国受众、内容定位及同龄历史表现；通过已记录的公开商务入口评估合作，不自动联系或推算报价。
-补录带来源的封面、开场、场景、结构和评论观察，未取得前不下内容因果结论。</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>未取得的材料不分析；人工备注与系统直接读取指标分开。
-候选清单包含已收录非排除内容，逐条标注合作状态与市场；不自动计入已确认合作。
-高播放不等于高转化，不推断订单、销售额、ROI或合作费用。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=demoNEW0001</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>[DEMO] Yozma IN-10 Pro review</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>高播放视频</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>本周新上线</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>明确合作</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>高播放视频；本周发布；合作状态：明确合作。
-最后有效展示快照：2026-10-26T06:00:00+00:00，播放 80,000，点赞 100，评论 10，分享 不可用。
-达到 YouTube / YouTube 普通视频 的高播放阈值 50,000。
-同龄样本 0 条；样本不足/格式未知/缺少同龄快照，不计算精确倍数。
-增长速度不可用：尚无有效的两次观测窗口，累计播放不视为本周新增。</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>原标题：[DEMO] Yozma IN-10 Pro review
-原标题品牌词：Yozma；车型词：IN-10 Pro。
-归纳主题标签（不等于原标题原词）：评测。</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>无附加推测</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">封面：不可用，未取得对应材料  
-开场：不可用，未取得对应材料  
-测试场景：不可用，未取得对应材料  
-内容结构：不可用，未取得对应材料  
-观众讨论点：不可用，未取得对应材料  
-字幕/口播：不可用，未取得对应材料  </t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>目前只满足绝对高播放标准，尚不足以认定相对账号表现异常。现有指标不能证明传播原因、自然流量比例或转化效果。</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Qronge选题验证：以适用人群、实际体验和优缺点清单组织评测，先复核原片的评测维度。
-创作者机会：复核 DEMO测试账号 的美国受众、内容定位及同龄历史表现；通过已记录的公开商务入口评估合作，不自动联系或推算报价。
-补齐同账号最近10–12条同形式视频的同龄快照，再判断是否相对爆款。
-补录带来源的封面、开场、场景、结构和评论观察，未取得前不下内容因果结论。</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>未取得的材料不分析；人工备注与系统直接读取指标分开。
-候选清单包含已收录非排除内容，逐条标注合作状态与市场；不自动计入已确认合作。
-高播放不等于高转化，不推断订单、销售额、ROI或合作费用。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:N3"/>
+  <autoFilter ref="A1:A4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2954,7 +2387,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -2987,10 +2420,8 @@
           <t>demo, tuttio, soleil01, gb, pro, off-road, first, ride</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>不可用</t>
-        </is>
+      <c r="P2" t="n">
+        <v>2500</v>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
@@ -3071,7 +2502,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -3359,7 +2790,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -3392,10 +2823,8 @@
           <t>demo, tuttio, soleil01, gb, pro, off-road, first, ride</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>不可用</t>
-        </is>
+      <c r="P2" t="n">
+        <v>2500</v>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
@@ -3476,7 +2905,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -3595,7 +3024,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T02:27:13.868992+00:00</t>
+          <t>2026-10-30T02:55:55.458653+00:00</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -3629,7 +3058,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>400</v>
+        <v>4000</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
@@ -4289,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -4597,7 +4026,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>first_observed_creators</t>
+          <t>excluded_low_views</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -4607,27 +4036,47 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>cross_platform_creators</t>
+          <t>excluded_unknown_views</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>first_observed_creators</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>cross_platform_creators</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>口径</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>多标签占比可超过100%；跨平台播放量未去重受众</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B31"/>
+  <autoFilter ref="A1:B33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4737,34 +4186,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="60" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>原视频</t>
+          <t>视频</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -4774,94 +4209,24 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>品牌</t>
+          <t>数据</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>车型</t>
+          <t>关键词</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>红人</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>平台</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>发布时间</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>播放</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>高播放</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>相对爆款</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>基线样本</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>同龄中位数</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>倍数</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>置信度</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>增长每天</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>依据</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>分析材料</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>事实与推测</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Qronge行动</t>
+          <t>内容方向</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=demoNEW0001</t>
+          <t>https://www.youtube.com/watch?v=demoREL0001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -4871,86 +4236,24 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Yozma</t>
+          <t>播放 4,000；赞 100；评 10；分享 不可用；同龄基线 4倍；快照 2026-10-16T07:00:00+00:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>IN-10 Pro</t>
+          <t>demo, yozma, in-10, pro, review</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>DEMO测试账号</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19T08:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>80000</v>
-      </c>
-      <c r="I2" t="b">
-        <v>1</v>
-      </c>
-      <c r="J2" t="b">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>不可用</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>不可用</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>样本不足/格式未知/缺少同龄快照</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>不可用</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>累计播放达到阈值 50,000；</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>标题, 描述</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>研究标题中的“demo / yozma / in-10 / pro / review”表达，并人工核查原视频测试条件；尚不能判断转化。</t>
+          <t>评测</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=demoREL0001</t>
+          <t>https://www.youtube.com/watch?v=demoNEW0001</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -4960,80 +4263,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Yozma</t>
+          <t>播放 80,000；赞 100；评 10；分享 不可用；快照 2026-10-26T06:00:00+00:00</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>IN-10 Pro</t>
+          <t>demo, yozma, in-10, pro, review</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>DEMO同龄样本账号</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09T07:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>400</v>
-      </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>10</v>
-      </c>
-      <c r="L3" t="n">
-        <v>100</v>
-      </c>
-      <c r="M3" t="n">
-        <v>4</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>同龄样本充分</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>不可用</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>同账号同形式同龄中位数的 4.0 倍；</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>标题, 描述</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>研究标题中的“demo / yozma / in-10 / pro / review”表达，并人工核查原视频测试条件；尚不能判断转化。</t>
+          <t>评测</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S3"/>
+  <autoFilter ref="A1:E3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>